<commit_message>
Mô tả thay đổi
</commit_message>
<xml_diff>
--- a/TKH_SYSTEM/frontend/templates/student-import-template.xlsx
+++ b/TKH_SYSTEM/frontend/templates/student-import-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phat.ngo\Desktop\TKH PROJECT\TKH_SYSTEM\frontend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1773A35-D17E-408F-95E1-56B14CE89446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB45F03A-C863-4334-AA70-317122D7217A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B114F50D-8FFF-43C7-8BA5-DFD0ACB85915}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="28">
   <si>
     <t>Giới tính</t>
   </si>
@@ -65,14 +65,71 @@
     <t>Ti-mô-thê</t>
   </si>
   <si>
-    <t>Họ và Tên</t>
+    <t>Nguyễn Văn 3</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 4</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 5</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 6</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 7</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 8</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 9</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 10</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn 11</t>
+  </si>
+  <si>
+    <t>Nữ</t>
+  </si>
+  <si>
+    <t>Họ và tên</t>
+  </si>
+  <si>
+    <t>Trịnh Thiên Phú</t>
+  </si>
+  <si>
+    <t>Nê-hê-mi</t>
+  </si>
+  <si>
+    <t>Phạm Bá Nam</t>
+  </si>
+  <si>
+    <t>Ma-ry</t>
+  </si>
+  <si>
+    <t>Ca-lép</t>
+  </si>
+  <si>
+    <t>Sa-ra</t>
+  </si>
+  <si>
+    <t>Giô-na-than</t>
+  </si>
+  <si>
+    <t>Giê-rê-mi</t>
+  </si>
+  <si>
+    <t>Ê-xơ-ra</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +141,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -448,10 +511,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD6E91B3-A24A-4522-89E5-76E2987A12D6}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="3" max="3" width="12.88671875" customWidth="1"/>
     <col min="4" max="4" width="15.44140625" customWidth="1"/>
     <col min="5" max="5" width="16.109375" customWidth="1"/>
@@ -459,7 +522,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -476,7 +539,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -488,10 +551,198 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
         <v>7</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="1">
+        <v>35777</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="D2" numberStoredAsText="1"/>

</xml_diff>